<commit_message>
feat: Nang cap toan dien tieu de cot tieng Viet va tu dong can rong cot trong cac file mau Excel, CSV, Word
</commit_message>
<xml_diff>
--- a/Du_Lieu_Mau_He_Thong/1_File_Excel_XLSX/Bang_bieu_phi_dich_vu_the_va_tai_khoan_2026.xlsx
+++ b/Du_Lieu_Mau_He_Thong/1_File_Excel_XLSX/Bang_bieu_phi_dich_vu_the_va_tai_khoan_2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataSheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,10 +33,10 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="10"/>
+      <sz val="10.5"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0000843D"/>
         <bgColor rgb="0000843D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F9F5"/>
+        <bgColor rgb="00F4F9F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,13 +82,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,27 +467,27 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="51" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dịch vụ tài khoản &amp; thẻ</t>
+          <t>Dịch vụ tài khoản &amp; thẻ thanh toán</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Mức phí chuẩn (VND)</t>
+          <t>Mức phí tiêu chuẩn (VND)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Ưu đãi khách hàng Digibank</t>
+          <t>Ưu đãi trên VCB Digibank</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -482,188 +497,174 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Ghi chú quy định</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Mở tài khoản thanh toán VND</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mở tại quầy giao dịch hoặc eKYC trực tuyến</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Duy trì số dư tài khoản tối thiểu</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>0 VND</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>0 VND</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Không yêu cầu duy trì số dư</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Phát hành thẻ ghi nợ Vietcombank Connect24</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Miễn phí khi mở online</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Mở tại quầy hoặc eKYC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Duy trì số dư tài khoản tối thiểu</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Không yêu cầu số dư</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Phát hành thẻ ghi nợ Vietcombank Connect24</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>50,000 VND</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Miễn phí khi mở online</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Thẻ chip không tiếp xúc Contactless</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Rút tiền tại cây ATM cùng hệ thống VCB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1,100 VND / GD</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Thẻ chip Contactless</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Rút tiền tại ATM cùng hệ thống Vietcombank</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>1,100 VND / GD</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>1,100 VND / GD</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Đã bao gồm thuế GTGT (VAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Rút tiền tại cây ATM ngoài hệ thống (Napas)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>3300</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>3,300 VND / GD</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Đã bao gồm VAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Rút tiền tại ATM ngân hàng khác (Napas)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>3,300 VND / GD</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>3,300 VND / GD</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Đã bao gồm thuế GTGT (VAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Chuyển tiền trong và ngoài hệ thống VCB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Miễn phí trọn đời</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Đã bao gồm VAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Chuyển tiền trong &amp; ngoài hệ thống VCB</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>0 VND</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Miễn phí trọn đời trên Digibank</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Áp dụng cho mọi giao dịch trên Digibank</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Quản lý tài khoản không hoạt động (&gt;12 tháng)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>30,000 VND / tháng</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>30,000 VND / tháng</t>
-        </is>
-      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Miễn phí</t>
@@ -671,7 +672,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Chỉ thu khi tài khoản còn số dư</t>
+          <t>Chỉ thu khi tài khoản còn số dư dương</t>
         </is>
       </c>
     </row>

</xml_diff>